<commit_message>
Renommage partie corps du modèle métier b97fd8107d5fdff5237894bebe54d4003b3fe9f2
</commit_message>
<xml_diff>
--- a/htr-Corps-ModeleMetier/ig/mappingPrescriptionCDAFHIR.xlsx
+++ b/htr-Corps-ModeleMetier/ig/mappingPrescriptionCDAFHIR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="43">
   <si>
     <t>Property</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-13T08:32:48+00:00</t>
+    <t>2025-10-21T08:19:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -135,13 +135,16 @@
     <t>inFulfillmentOf.order.ps3-20:accessionNumber</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/uv/fhir-clinical-document/StructureDefinition/OrderExtension</t>
-  </si>
-  <si>
-    <t>extension:OrderExtension</t>
-  </si>
-  <si>
-    <t>extension:OrderExtension.ValueReference.ServiceRequest.identifier</t>
+    <t>http://hl7.org/fhir/StructureDefinition/event-basedOn</t>
+  </si>
+  <si>
+    <t>extension:basedOn</t>
+  </si>
+  <si>
+    <t>extension:basedOnExtension.ValueReference.ServiceRequest.identifier</t>
+  </si>
+  <si>
+    <t>extension:basedOn.ValueReference.ServiceRequest.identifier</t>
   </si>
 </sst>
 </file>
@@ -552,7 +555,7 @@
         <v>33</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" s="2"/>
     </row>

</xml_diff>